<commit_message>
Finalised prior to shipment, customer FW yet finalised
</commit_message>
<xml_diff>
--- a/PCBA/TesterSpecific/FRU PROGRAMMING TOOLKIT/Data/Excel File/FRU Array.xlsx
+++ b/PCBA/TesterSpecific/FRU PROGRAMMING TOOLKIT/Data/Excel File/FRU Array.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Emerson\FRU Programming Excel\Try Changing all to 32 Target Page Size\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23C1E02F-19CA-4A52-9EEF-7456DD32A8DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2E28E79-3521-4DC5-ABCE-C602EAB9DFC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -107,21 +107,12 @@
     <t>Model Revision</t>
   </si>
   <si>
-    <t>0056</t>
-  </si>
-  <si>
     <t>FW Major Rev</t>
   </si>
   <si>
-    <t>0058</t>
-  </si>
-  <si>
     <t>MCU FW Minor Rev</t>
   </si>
   <si>
-    <t>005A</t>
-  </si>
-  <si>
     <t>Lifetime Turn On Time</t>
   </si>
   <si>
@@ -315,6 +306,15 @@
   </si>
   <si>
     <t>02A7</t>
+  </si>
+  <si>
+    <t>003C</t>
+  </si>
+  <si>
+    <t>003E</t>
+  </si>
+  <si>
+    <t>0040</t>
   </si>
 </sst>
 </file>
@@ -745,10 +745,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A6" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C6" s="5">
         <v>65</v>
@@ -790,10 +790,10 @@
         <v>22</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D9">
         <v>32</v>
@@ -804,7 +804,7 @@
         <v>23</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>24</v>
+        <v>91</v>
       </c>
       <c r="C10" s="2">
         <v>4141</v>
@@ -815,10 +815,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>9</v>
@@ -829,10 +829,10 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>28</v>
+        <v>93</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>9</v>
@@ -843,13 +843,13 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D13">
         <v>32</v>
@@ -857,13 +857,13 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A14" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D14">
         <v>32</v>
@@ -871,13 +871,13 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A15" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D15">
         <v>32</v>
@@ -885,10 +885,10 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A16" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C16" s="2">
         <v>3700</v>
@@ -899,10 +899,10 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A17" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C17" s="2">
         <v>1400</v>
@@ -913,10 +913,10 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A18" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C18" s="2">
         <v>78000000</v>
@@ -927,13 +927,13 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A19" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D19">
         <v>32</v>
@@ -941,10 +941,10 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A20" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>18</v>
@@ -955,10 +955,10 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A21" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>6</v>
@@ -969,10 +969,10 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A22" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>6</v>
@@ -983,10 +983,10 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A23" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>10</v>
@@ -997,13 +997,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A24" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D24">
         <v>32</v>
@@ -1011,10 +1011,10 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A25" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>6</v>
@@ -1025,13 +1025,13 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A26" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D26">
         <v>32</v>
@@ -1039,10 +1039,10 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A27" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>6</v>
@@ -1053,13 +1053,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A28" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D28">
         <v>32</v>
@@ -1067,10 +1067,10 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A29" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>6</v>
@@ -1081,10 +1081,10 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A30" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>6</v>
@@ -1095,10 +1095,10 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A31" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>6</v>
@@ -1109,10 +1109,10 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A32" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>13</v>
@@ -1123,13 +1123,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A33" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D33">
         <v>32</v>
@@ -1137,13 +1137,13 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A34" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D34">
         <v>32</v>
@@ -1151,13 +1151,13 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A35" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D35">
         <v>32</v>
@@ -1165,13 +1165,13 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A36" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D36">
         <v>32</v>
@@ -1179,13 +1179,13 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A37" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D37">
         <v>32</v>
@@ -1193,13 +1193,13 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A38" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D38">
         <v>32</v>
@@ -1207,13 +1207,13 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A39" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D39">
         <v>32</v>
@@ -1221,13 +1221,13 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A40" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D40">
         <v>32</v>

</xml_diff>